<commit_message>
fix(diagram-converter): retain pivot items for Excel refresh
Refs #2880

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/diagram-converter/core/src/main/resources/MigrationAnalyzerResultTemplate.xlsx
+++ b/diagram-converter/core/src/main/resources/MigrationAnalyzerResultTemplate.xlsx
@@ -6010,13 +6010,22 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending"/>
+    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="5"/>
   </rowFields>
+  <rowItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colItems count="1">
     <i/>
   </colItems>
@@ -6093,7 +6102,11 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D7F6E40E-66E4-C54C-BE9C-B416373A68C9}" name="PivotTable6" cacheId="98" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" multipleFieldFilters="0" chartFormat="2" rowHeaderCaption="Filename">
   <location ref="K25:L71" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="8">
-    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending"/>
+    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -6105,6 +6118,11 @@
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
+  <rowItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colItems count="1">
     <i/>
   </colItems>
@@ -6173,7 +6191,11 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending"/>
+    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -6182,6 +6204,11 @@
   <rowFields count="1">
     <field x="3"/>
   </rowFields>
+  <rowItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colItems count="1">
     <i/>
   </colItems>
@@ -6262,7 +6289,11 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending"/>
+    <pivotField axis="axisRow" dataField="1" compact="0" outline="0" showAll="0" sortType="ascending">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -6270,6 +6301,11 @@
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
+  <rowItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colFields count="1">
     <field x="-2"/>
   </colFields>
@@ -6418,9 +6454,21 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="1">
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="3">
@@ -6428,6 +6476,11 @@
     <field x="5"/>
     <field x="6"/>
   </rowFields>
+  <rowItems count="1">
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colItems count="1">
     <i/>
   </colItems>

</xml_diff>